<commit_message>
rag ragas평가 및 rrf 비율 1:1로 변경
</commit_message>
<xml_diff>
--- a/rag/eval/ragas_dataset.xlsx
+++ b/rag/eval/ragas_dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\00project\SKN20-FINAL-2TEAM\rag\eval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45BD6162-FD06-4055-A852-CB3410E37D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D4C7299-113E-4AD3-A32D-95E37C68268A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="960" windowWidth="13944" windowHeight="12000" xr2:uid="{B263BCC5-AE7D-4EF2-9AB3-8302F8AAA892}"/>
+    <workbookView xWindow="5040" yWindow="1104" windowWidth="12468" windowHeight="10500" xr2:uid="{B263BCC5-AE7D-4EF2-9AB3-8302F8AAA892}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,13 +36,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="95">
   <si>
     <t>user_query</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>10-2006-0001051</t>
   </si>
   <si>
     <t>apply_num_1</t>
@@ -514,6 +511,14 @@
   </si>
   <si>
     <t>apply_num_2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10-2006-0001051</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10-2015-0102997</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -975,16 +980,16 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.4" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="39.6" x14ac:dyDescent="0.4">
@@ -992,13 +997,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1</v>
+        <v>94</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>1</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="39.6" x14ac:dyDescent="0.4">
@@ -1006,13 +1011,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="52.8" x14ac:dyDescent="0.4">
@@ -1020,10 +1025,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="39.6" x14ac:dyDescent="0.4">
@@ -1031,10 +1036,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="66" x14ac:dyDescent="0.4">
@@ -1042,13 +1047,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="52.8" x14ac:dyDescent="0.4">
@@ -1056,13 +1061,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="52.8" x14ac:dyDescent="0.4">
@@ -1070,13 +1075,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="52.8" x14ac:dyDescent="0.4">
@@ -1084,13 +1089,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="66" x14ac:dyDescent="0.4">
@@ -1098,19 +1103,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="66" x14ac:dyDescent="0.4">
@@ -1118,13 +1123,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="79.2" x14ac:dyDescent="0.4">
@@ -1132,13 +1137,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="52.8" x14ac:dyDescent="0.4">
@@ -1146,16 +1151,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="52.8" x14ac:dyDescent="0.4">
@@ -1163,13 +1168,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="52.8" x14ac:dyDescent="0.4">
@@ -1177,13 +1182,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
@@ -1191,10 +1196,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
@@ -1202,13 +1207,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
@@ -1216,13 +1221,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
@@ -1230,13 +1235,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
@@ -1244,13 +1249,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="E20" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="66" x14ac:dyDescent="0.3">
@@ -1258,10 +1263,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
@@ -1269,13 +1274,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="66" x14ac:dyDescent="0.3">
@@ -1283,10 +1288,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
@@ -1294,13 +1299,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
@@ -1308,10 +1313,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
@@ -1319,10 +1324,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
@@ -1330,10 +1335,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
@@ -1341,10 +1346,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
@@ -1352,13 +1357,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="79.2" x14ac:dyDescent="0.3">
@@ -1366,13 +1371,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
@@ -1380,10 +1385,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
@@ -1391,10 +1396,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="52.8" x14ac:dyDescent="0.3">
@@ -1402,10 +1407,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
@@ -1413,10 +1418,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="52.8" x14ac:dyDescent="0.3">
@@ -1424,10 +1429,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="52.8" x14ac:dyDescent="0.3">
@@ -1435,10 +1440,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>